<commit_message>
Atualização automática da planilha
</commit_message>
<xml_diff>
--- a/template-softexpert.xlsx
+++ b/template-softexpert.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30516"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://planoeplano.sharepoint.com/sites/Softexpert/Documentos Compartilhados/Status Report - Executivo/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1991" documentId="11_C24A341F8ED520438A3C56126D326013BF438F93" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{57A372C9-D2C4-434A-8F3F-F808BDA48EB8}"/>
+  <xr:revisionPtr revIDLastSave="1996" documentId="11_C24A341F8ED520438A3C56126D326013BF438F93" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0D07A907-3234-4FF4-AACF-4DEF83992DC1}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="500" firstSheet="8" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2312,7 +2312,7 @@
       </c>
       <c r="B4" s="8" t="str">
         <f ca="1">TEXT(NOW(),"DD/MM/AAAA")</f>
-        <v>24/08/2026</v>
+        <v>22/09/2026</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="15" customHeight="1">
@@ -9049,6 +9049,7 @@
     <col min="5" max="11" width="12.28515625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="13" customWidth="1"/>
     <col min="13" max="13" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="14.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="15" customHeight="1">
@@ -9195,7 +9196,9 @@
       <c r="M3" s="70">
         <v>19810</v>
       </c>
-      <c r="N3" s="70"/>
+      <c r="N3" s="70">
+        <v>19810</v>
+      </c>
       <c r="O3" s="70"/>
       <c r="P3" s="70"/>
       <c r="Q3" s="70"/>
@@ -9302,7 +9305,9 @@
       <c r="M6" s="70">
         <v>5260</v>
       </c>
-      <c r="N6" s="70"/>
+      <c r="N6" s="70">
+        <v>5260</v>
+      </c>
       <c r="O6" s="70"/>
       <c r="P6" s="70"/>
       <c r="Q6" s="70"/>
@@ -9451,7 +9456,9 @@
       <c r="M11" s="70">
         <v>209292.75</v>
       </c>
-      <c r="N11" s="70"/>
+      <c r="N11" s="70">
+        <v>80155</v>
+      </c>
       <c r="O11" s="70"/>
       <c r="P11" s="70"/>
       <c r="Q11" s="70"/>
@@ -9506,7 +9513,7 @@
       </c>
       <c r="B16" s="76">
         <f>SUM(E3:Q13)</f>
-        <v>1069155.4300000002</v>
+        <v>1174380.43</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="15" customHeight="1">
@@ -9515,7 +9522,7 @@
       </c>
       <c r="B17" s="78">
         <f>B15-B16</f>
-        <v>898177.56999999983</v>
+        <v>792952.57000000007</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="14.25" customHeight="1"/>
@@ -9533,12 +9540,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="25b7c34c-a120-4ac3-ab60-c6bebc005a32">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="2aea894b-94ad-406a-ad4e-500caf6a56d3" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -9737,18 +9746,16 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="25b7c34c-a120-4ac3-ab60-c6bebc005a32">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="2aea894b-94ad-406a-ad4e-500caf6a56d3" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B2FB2B9C-EC1C-4F74-BCCE-02A14630346E}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{07A6E785-FFA4-4B45-919B-A658CFA9E29F}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -9756,5 +9763,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{07A6E785-FFA4-4B45-919B-A658CFA9E29F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B2FB2B9C-EC1C-4F74-BCCE-02A14630346E}"/>
 </file>
</xml_diff>